<commit_message>
Add HSK2 tab to HSK_words.xlsx
</commit_message>
<xml_diff>
--- a/HSK_words.xlsx
+++ b/HSK_words.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="HSK1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="HSK2" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4936,4 +4937,4535 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C301"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Chữ Trung Quốc</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>啊</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%95%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>安</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>般</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%88%AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>板</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9D%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>办</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8A%9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>饱</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A5%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>报</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8A%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>背</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%83%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>笔</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AC%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>必</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BF%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>变</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>便</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BE%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>遍</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%81%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>表</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A1%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>部</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%83%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>才</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>参</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>餐</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A4%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>草</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%8D%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>层</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B1%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>查</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9F%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>长</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%95%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>超</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B6%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>晨</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%99%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>称</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A7%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>成</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%88%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>楚</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A5%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>处</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>船</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%88%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>吹</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>春</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%98%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>词</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AF%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>带</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B8%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>单</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8D%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>但</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BD%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>当</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BD%93</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>倒</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%80%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>灯</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%81%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BD%8E</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>典</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>掉</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8E%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>定</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>冬</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%86%AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>懂</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%87%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>度</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BA%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>短</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9F%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>段</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AE%B5</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>队</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%98%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>而</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%80%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>发</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>法</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>51</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B3%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>份</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>52</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>封</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>53</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B0%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>复</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>54</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>该</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>55</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AF%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>改</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>56</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%94%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>感</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>57</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%84%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>刚</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>58</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>更</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>59</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9B%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>公</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>60</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>共</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>61</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>狗</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>62</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8B%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>够</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>63</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>故</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>64</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%95%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>顾</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>65</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A1%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>观</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>66</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A7%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>惯</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>67</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%83%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>广</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>68</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B9%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>海</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>69</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B5%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>喊</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>70</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%96%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>合</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>71</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>河</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>72</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B2%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>黑</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>73</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%BB%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>红</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>74</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BA%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>忽</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>75</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BF%BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>湖</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>76</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B9%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>护</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>77</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8A%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>划</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>78</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>画</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>79</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%94%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>换</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>80</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8D%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>黄</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>81</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%BB%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>活</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>82</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B4%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>或</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>83</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%88%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>级</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>84</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BA%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>急</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>85</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%80%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>己</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>86</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B7%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>计</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>87</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AE%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>际</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>88</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%99%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>绩</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>89</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>加</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>90</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8A%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>检</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>91</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A3%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>件</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>92</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>健</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>93</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%81%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>讲</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>94</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AE%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>交</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>95</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>角</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>96</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A7%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>饺</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>97</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A5%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>脚</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>98</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%84%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>接</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>99</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8E%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>街</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>100</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A1%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>节</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>101</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%8A%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>结</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>102</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%93</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>借</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>103</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%80%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>斤</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>104</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%96%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>近</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>105</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BF%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>经</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>106</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>睛</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>107</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9D%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>静</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>108</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%9D%99</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>久</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>109</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B9%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>酒</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>110</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%85%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>举</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>111</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>句</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>112</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>卡</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>113</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8D%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>康</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>114</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BA%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>靠</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>115</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%9D%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>科</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>116</v>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A7%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>可</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>117</v>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>克</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>118</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>刻</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>119</v>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>空</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>120</v>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A9%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>哭</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>121</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%93%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>筷</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>122</v>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AD%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>拉</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>123</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8B%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>蓝</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>124</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%93%9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>篮</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>125</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AF%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>乐</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>126</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B9%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>离</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>127</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A6%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>礼</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>128</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A4%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>理</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>129</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%90%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>力</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>130</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8A%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>利</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>131</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>例</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>132</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BE%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>脸</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>133</v>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%84%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>练</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>134</v>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>凉</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>135</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%87%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>亮</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>136</v>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>辆</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>137</v>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BE%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>量</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>138</v>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%87%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>留</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>139</v>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%95%99</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>流</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>140</v>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B5%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>旅</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>141</v>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%97%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>绿</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>142</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>论</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>143</v>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AE%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>卖</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>144</v>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8D%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>满</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>145</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%BB%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>猫</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>146</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8C%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>末</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>147</v>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9C%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>目</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>148</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9B%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>鸟</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>149</v>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%B8%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>弄</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>150</v>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BC%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>努</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>151</v>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8A%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>爬</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>152</v>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%88%AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>怕</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>153</v>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%80%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>排</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>154</v>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8E%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>碰</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>155</v>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A2%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>篇</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>156</v>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AF%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>片</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>157</v>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%89%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>漂</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>158</v>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%BC%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>平</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>159</v>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B9%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>瓶</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>160</v>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%93%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>普</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>161</v>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%99%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>其</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>162</v>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>骑</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>163</v>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%AA%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>千</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>164</v>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8D%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>墙</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>165</v>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A2%99</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>且</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>166</v>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>青</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>167</v>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%9D%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>轻</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>168</v>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BD%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>清</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>169</v>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B8%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>情</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>170</v>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%83%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>晴</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>171</v>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%99%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>秋</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>172</v>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A7%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>求</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>173</v>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B1%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>取</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>174</v>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>全</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>175</v>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>确</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>176</v>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A1%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>然</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>177</v>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%84%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>让</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>178</v>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AE%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>如</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>179</v>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A6%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>入</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>180</v>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>色</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>181</v>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%89%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>声</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>182</v>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A3%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>省</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>183</v>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9C%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>实</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>184</v>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>食</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>185</v>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A3%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>使</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>186</v>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BD%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>示</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>187</v>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A4%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>市</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>188</v>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B8%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>适</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>189</v>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%80%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>室</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>190</v>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>收</t>
+        </is>
+      </c>
+      <c r="B192" t="n">
+        <v>191</v>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%94%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>受</t>
+        </is>
+      </c>
+      <c r="B193" t="n">
+        <v>192</v>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>舒</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>193</v>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%88%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>熟</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>194</v>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%86%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>数</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>195</v>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%95%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>顺</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>196</v>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A1%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>司</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>197</v>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>思</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>198</v>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%80%9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>算</t>
+        </is>
+      </c>
+      <c r="B200" t="n">
+        <v>199</v>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AE%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>虽</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>200</v>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%99%BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>随</t>
+        </is>
+      </c>
+      <c r="B202" t="n">
+        <v>201</v>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%9A%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>所</t>
+        </is>
+      </c>
+      <c r="B203" t="n">
+        <v>202</v>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>它</t>
+        </is>
+      </c>
+      <c r="B204" t="n">
+        <v>203</v>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>态</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>204</v>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%80%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>堂</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>205</v>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A0%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>讨</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>206</v>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AE%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>套</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>207</v>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A5%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>特</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>208</v>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%89%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>疼</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>209</v>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%96%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>提</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
+        <v>210</v>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8F%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>题</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>211</v>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A2%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>铁</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>212</v>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%93%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>庭</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>213</v>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BA%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>停</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>214</v>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%81%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>挺</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>215</v>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8C%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>通</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>216</v>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%80%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>头</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>217</v>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>推</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>218</v>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8E%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>腿</t>
+        </is>
+      </c>
+      <c r="B220" t="n">
+        <v>219</v>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%85%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>完</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>220</v>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>碗</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>221</v>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A2%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>万</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>222</v>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>王</t>
+        </is>
+      </c>
+      <c r="B224" t="n">
+        <v>223</v>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8E%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>往</t>
+        </is>
+      </c>
+      <c r="B225" t="n">
+        <v>224</v>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BE%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>为</t>
+        </is>
+      </c>
+      <c r="B226" t="n">
+        <v>225</v>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>位</t>
+        </is>
+      </c>
+      <c r="B227" t="n">
+        <v>226</v>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BD%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>味</t>
+        </is>
+      </c>
+      <c r="B228" t="n">
+        <v>227</v>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%91%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>喂</t>
+        </is>
+      </c>
+      <c r="B229" t="n">
+        <v>228</v>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%96%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>温</t>
+        </is>
+      </c>
+      <c r="B230" t="n">
+        <v>229</v>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B8%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>闻</t>
+        </is>
+      </c>
+      <c r="B231" t="n">
+        <v>230</v>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%97%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>务</t>
+        </is>
+      </c>
+      <c r="B232" t="n">
+        <v>231</v>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8A%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>物</t>
+        </is>
+      </c>
+      <c r="B233" t="n">
+        <v>232</v>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%89%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>夏</t>
+        </is>
+      </c>
+      <c r="B234" t="n">
+        <v>233</v>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>相</t>
+        </is>
+      </c>
+      <c r="B235" t="n">
+        <v>234</v>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9B%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>响</t>
+        </is>
+      </c>
+      <c r="B236" t="n">
+        <v>235</v>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%93%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>向</t>
+        </is>
+      </c>
+      <c r="B237" t="n">
+        <v>236</v>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>像</t>
+        </is>
+      </c>
+      <c r="B238" t="n">
+        <v>237</v>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%83%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>鞋</t>
+        </is>
+      </c>
+      <c r="B239" t="n">
+        <v>238</v>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%9E%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>心</t>
+        </is>
+      </c>
+      <c r="B240" t="n">
+        <v>239</v>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BF%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>信</t>
+        </is>
+      </c>
+      <c r="B241" t="n">
+        <v>240</v>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BF%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>姓</t>
+        </is>
+      </c>
+      <c r="B242" t="n">
+        <v>241</v>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A7%93</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>须</t>
+        </is>
+      </c>
+      <c r="B243" t="n">
+        <v>242</v>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A1%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>许</t>
+        </is>
+      </c>
+      <c r="B244" t="n">
+        <v>243</v>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AE%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>选</t>
+        </is>
+      </c>
+      <c r="B245" t="n">
+        <v>244</v>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%80%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>雪</t>
+        </is>
+      </c>
+      <c r="B246" t="n">
+        <v>245</v>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%9B%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>言</t>
+        </is>
+      </c>
+      <c r="B247" t="n">
+        <v>246</v>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A8%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>颜</t>
+        </is>
+      </c>
+      <c r="B248" t="n">
+        <v>247</v>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A2%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>眼</t>
+        </is>
+      </c>
+      <c r="B249" t="n">
+        <v>248</v>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9C%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>阳</t>
+        </is>
+      </c>
+      <c r="B250" t="n">
+        <v>249</v>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%98%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>养</t>
+        </is>
+      </c>
+      <c r="B251" t="n">
+        <v>250</v>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>药</t>
+        </is>
+      </c>
+      <c r="B252" t="n">
+        <v>251</v>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%8D%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>业</t>
+        </is>
+      </c>
+      <c r="B253" t="n">
+        <v>252</v>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>夜</t>
+        </is>
+      </c>
+      <c r="B254" t="n">
+        <v>253</v>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>宜</t>
+        </is>
+      </c>
+      <c r="B255" t="n">
+        <v>254</v>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>已</t>
+        </is>
+      </c>
+      <c r="B256" t="n">
+        <v>255</v>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B7%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>以</t>
+        </is>
+      </c>
+      <c r="B257" t="n">
+        <v>256</v>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>椅</t>
+        </is>
+      </c>
+      <c r="B258" t="n">
+        <v>257</v>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A4%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>亿</t>
+        </is>
+      </c>
+      <c r="B259" t="n">
+        <v>258</v>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>意</t>
+        </is>
+      </c>
+      <c r="B260" t="n">
+        <v>259</v>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%84%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>因</t>
+        </is>
+      </c>
+      <c r="B261" t="n">
+        <v>260</v>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9B%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>阴</t>
+        </is>
+      </c>
+      <c r="B262" t="n">
+        <v>261</v>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%98%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>音</t>
+        </is>
+      </c>
+      <c r="B263" t="n">
+        <v>262</v>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%9F%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>银</t>
+        </is>
+      </c>
+      <c r="B264" t="n">
+        <v>263</v>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%93%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>印</t>
+        </is>
+      </c>
+      <c r="B265" t="n">
+        <v>264</v>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8D%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>应</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>265</v>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BA%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>英</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>266</v>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%8B%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>迎</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>267</v>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BF%8E</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>永</t>
+        </is>
+      </c>
+      <c r="B269" t="n">
+        <v>268</v>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B0%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>由</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>269</v>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%94%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>油</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>270</v>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B2%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>游</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>271</v>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B8%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>又</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>272</v>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>于</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>273</v>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%8E</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>鱼</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>274</v>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%B1%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>育</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>275</v>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%82%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>园</t>
+        </is>
+      </c>
+      <c r="B277" t="n">
+        <v>276</v>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9B%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>原</t>
+        </is>
+      </c>
+      <c r="B278" t="n">
+        <v>277</v>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8E%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>愿</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>278</v>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%84%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>越</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>279</v>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B6%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>云</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>280</v>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>运</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>281</v>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BF%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>咱</t>
+        </is>
+      </c>
+      <c r="B283" t="n">
+        <v>282</v>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%92%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>脏</t>
+        </is>
+      </c>
+      <c r="B284" t="n">
+        <v>283</v>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%84%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>澡</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>284</v>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%BE%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>占</t>
+        </is>
+      </c>
+      <c r="B286" t="n">
+        <v>285</v>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8D%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>照</t>
+        </is>
+      </c>
+      <c r="B287" t="n">
+        <v>286</v>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%85%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>者</t>
+        </is>
+      </c>
+      <c r="B288" t="n">
+        <v>287</v>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%80%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>直</t>
+        </is>
+      </c>
+      <c r="B289" t="n">
+        <v>288</v>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9B%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>只</t>
+        </is>
+      </c>
+      <c r="B290" t="n">
+        <v>289</v>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>纸</t>
+        </is>
+      </c>
+      <c r="B291" t="n">
+        <v>290</v>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BA%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>钟</t>
+        </is>
+      </c>
+      <c r="B292" t="n">
+        <v>291</v>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%92%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>周</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>292</v>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%91%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>主</t>
+        </is>
+      </c>
+      <c r="B294" t="n">
+        <v>293</v>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>助</t>
+        </is>
+      </c>
+      <c r="B295" t="n">
+        <v>294</v>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8A%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>装</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>295</v>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A3%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>自</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>296</v>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%87%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>租</t>
+        </is>
+      </c>
+      <c r="B298" t="n">
+        <v>297</v>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A7%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>组</t>
+        </is>
+      </c>
+      <c r="B299" t="n">
+        <v>298</v>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>嘴</t>
+        </is>
+      </c>
+      <c r="B300" t="n">
+        <v>299</v>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%98%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>座</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>300</v>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BA%A7</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add HSK3 tab to HSK_words.xlsx
</commit_message>
<xml_diff>
--- a/HSK_words.xlsx
+++ b/HSK_words.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="HSK1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="HSK2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="HSK3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9468,4 +9469,4535 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C301"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Chữ Trung Quốc</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>按</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8C%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>把</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8A%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>搬</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%90%AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>保</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BF%9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>被</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A2%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>币</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B8%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>标</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A0%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>并</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B9%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>播</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%92%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>补</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A1%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>布</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B8%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>步</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AD%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>材</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9D%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>采</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%87%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>彩</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BD%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>曾</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9B%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>察</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AF%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>产</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>厂</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8E%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>朝</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9C%9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>吵</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%B5</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>衬</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A1%AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>城</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9F%8E</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>程</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A8%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>持</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8C%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>充</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>初</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>除</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%99%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>础</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A1%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>传</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BC%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>创</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>此</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AD%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>村</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9D%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>存</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AD%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>达</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BE%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>代</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>待</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BE%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>刀</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>导</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AF%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>底</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BA%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>调</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B0%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>订</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AE%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>断</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%96%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>顿</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A1%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>烦</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%83%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>反</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>范</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%8C%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>防</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%98%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>访</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AE%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>啡</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%95%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>费</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>51</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B4%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>丰</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>52</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>53</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>夫</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>54</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>福</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>55</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A6%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>父</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>56</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%88%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>付</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>57</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>负</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>58</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B4%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>富</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>59</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AF%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>概</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>60</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A6%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>赶</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>61</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B5%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>敢</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>62</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%95%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>格</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>63</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A0%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>各</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>64</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>根</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>65</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A0%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>功</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>66</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8A%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>姑</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>67</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A7%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>古</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>68</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>挂</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>69</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8C%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>怪</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>70</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%80%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>管</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>71</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AE%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>光</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>72</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>规</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>73</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A7%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>哈</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>74</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%93%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>害</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>75</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>何</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>76</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BD%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>互</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>77</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>华</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>78</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8D%8E</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>化</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>79</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8C%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>环</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>80</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8E%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>婚</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>81</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A9%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>积</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>82</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A7%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>基</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>83</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9F%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>及</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>84</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>极</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>85</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9E%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>集</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>86</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%9B%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>纪</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>87</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BA%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>技</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>88</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8A%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>济</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>89</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B5%8E</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>继</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>90</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>价</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>91</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>架</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>92</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9E%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>坚</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>93</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9D%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>简</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>94</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AE%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>建</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>95</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BB%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>将</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>96</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B0%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>蕉</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>97</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%95%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>较</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>98</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BE%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>解</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>99</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A7%A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>界</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>100</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%95%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>101</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%87%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>仅</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>102</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>尽</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>103</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B0%BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>紧</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>104</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%B4%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>精</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>105</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%B2%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>景</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>106</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%99%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>警</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>107</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AD%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>境</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>108</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A2%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>旧</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>109</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%97%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>救</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>110</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%95%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>具</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>111</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>剧</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>112</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%89%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>据</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>113</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8D%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>决</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>114</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%86%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>绝</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>115</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>咖</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>116</v>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%92%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>恐</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>117</v>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%81%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>苦</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>118</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%8B%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>裤</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>119</v>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A3%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>况</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>120</v>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%86%B5</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>困</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>121</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9B%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>浪</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>122</v>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B5%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>类</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>123</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%B1%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>李</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>124</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9D%8E</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>历</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>125</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8E%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>立</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>126</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AB%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>丽</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>127</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>连</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>128</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BF%9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>联</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>129</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%81%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>烈</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>130</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%83%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>领</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>131</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A2%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>另</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>132</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>龙</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>133</v>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%BE%99</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>录</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>134</v>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BD%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>乱</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>135</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B9%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>落</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>136</v>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%90%BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>麻</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>137</v>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%BA%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>冒</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>138</v>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%86%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>媒</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>139</v>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AA%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>每</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>140</v>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AF%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>美</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>141</v>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BE%8E</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>迷</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>142</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BF%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>民</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>143</v>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B0%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>命</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>144</v>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%91%BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>某</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>145</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9F%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>母</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>146</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AF%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>木</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>147</v>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9C%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>内</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>148</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%86%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>念</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>149</v>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BF%B5</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>娘</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>150</v>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A8%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>农</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>151</v>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%86%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>暖</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>152</v>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9A%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>拍</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>153</v>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8B%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>牌</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>154</v>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%89%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>派</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>155</v>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B4%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>判</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>156</v>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>胖</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>157</v>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%83%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>配</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>158</v>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%85%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>批</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>159</v>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>皮</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>160</v>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9A%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>啤</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>161</v>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%95%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>品</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>162</v>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%93%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>评</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>163</v>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AF%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>苹</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>164</v>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%8B%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>破</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>165</v>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A0%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>齐</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>166</v>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%BD%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>奇</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>167</v>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A5%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>器</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>168</v>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%99%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>强</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>169</v>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BC%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>桥</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>170</v>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A1%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>巧</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>171</v>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B7%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>切</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>172</v>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>亲</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>173</v>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>庆</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>174</v>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BA%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>区</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>175</v>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8C%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>缺</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>176</v>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BC%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>裙</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>177</v>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A3%99</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>群</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>178</v>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BE%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>任</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>179</v>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>仍</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>180</v>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>容</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>181</v>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>赛</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>182</v>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B5%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>散</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>183</v>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%95%A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>沙</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>184</v>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B2%99</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>衫</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>185</v>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A1%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>善</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>186</v>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%96%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>伤</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>187</v>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BC%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>设</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>188</v>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AE%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>社</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>189</v>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A4%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>深</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>190</v>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B7%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>神</t>
+        </is>
+      </c>
+      <c r="B192" t="n">
+        <v>191</v>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A5%9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>升</t>
+        </is>
+      </c>
+      <c r="B193" t="n">
+        <v>192</v>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8D%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>胜</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>193</v>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%83%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>失</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>194</v>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>石</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>195</v>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9F%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>始</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>196</v>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A7%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>世</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>197</v>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>198</v>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BC%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>似</t>
+        </is>
+      </c>
+      <c r="B200" t="n">
+        <v>199</v>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BC%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>势</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>200</v>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8A%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>首</t>
+        </is>
+      </c>
+      <c r="B202" t="n">
+        <v>201</v>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A6%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>输</t>
+        </is>
+      </c>
+      <c r="B203" t="n">
+        <v>202</v>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BE%93</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>属</t>
+        </is>
+      </c>
+      <c r="B204" t="n">
+        <v>203</v>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B1%9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>术</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>204</v>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9C%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>束</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>205</v>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9D%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>双</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>206</v>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>死</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>207</v>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AD%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>速</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>208</v>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%80%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>台</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>209</v>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>谈</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
+        <v>210</v>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B0%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>汤</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>211</v>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B1%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>糖</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>212</v>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%B3%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>甜</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>213</v>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%94%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>跳</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>214</v>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B7%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>痛</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>215</v>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%97%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>突</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>216</v>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AA%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>217</v>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9C%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>团</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>218</v>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9B%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>退</t>
+        </is>
+      </c>
+      <c r="B220" t="n">
+        <v>219</v>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%80%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>望</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>220</v>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9C%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>危</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>221</v>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8D%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>围</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>222</v>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9B%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>伟</t>
+        </is>
+      </c>
+      <c r="B224" t="n">
+        <v>223</v>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BC%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>卫</t>
+        </is>
+      </c>
+      <c r="B225" t="n">
+        <v>224</v>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8D%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>握</t>
+        </is>
+      </c>
+      <c r="B226" t="n">
+        <v>225</v>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8F%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>屋</t>
+        </is>
+      </c>
+      <c r="B227" t="n">
+        <v>226</v>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B1%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>武</t>
+        </is>
+      </c>
+      <c r="B228" t="n">
+        <v>227</v>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AD%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>舞</t>
+        </is>
+      </c>
+      <c r="B229" t="n">
+        <v>228</v>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%88%9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>误</t>
+        </is>
+      </c>
+      <c r="B230" t="n">
+        <v>229</v>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AF%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>希</t>
+        </is>
+      </c>
+      <c r="B231" t="n">
+        <v>230</v>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B8%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>戏</t>
+        </is>
+      </c>
+      <c r="B232" t="n">
+        <v>231</v>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%88%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>显</t>
+        </is>
+      </c>
+      <c r="B233" t="n">
+        <v>232</v>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%98%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>险</t>
+        </is>
+      </c>
+      <c r="B234" t="n">
+        <v>233</v>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%99%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>线</t>
+        </is>
+      </c>
+      <c r="B235" t="n">
+        <v>234</v>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BA%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>乡</t>
+        </is>
+      </c>
+      <c r="B236" t="n">
+        <v>235</v>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B9%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>香</t>
+        </is>
+      </c>
+      <c r="B237" t="n">
+        <v>236</v>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A6%99</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>箱</t>
+        </is>
+      </c>
+      <c r="B238" t="n">
+        <v>237</v>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AE%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>象</t>
+        </is>
+      </c>
+      <c r="B239" t="n">
+        <v>238</v>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B1%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>消</t>
+        </is>
+      </c>
+      <c r="B240" t="n">
+        <v>239</v>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B6%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>效</t>
+        </is>
+      </c>
+      <c r="B241" t="n">
+        <v>240</v>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%95%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>血</t>
+        </is>
+      </c>
+      <c r="B242" t="n">
+        <v>241</v>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A1%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>形</t>
+        </is>
+      </c>
+      <c r="B243" t="n">
+        <v>242</v>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BD%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>幸</t>
+        </is>
+      </c>
+      <c r="B244" t="n">
+        <v>243</v>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B9%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>性</t>
+        </is>
+      </c>
+      <c r="B245" t="n">
+        <v>244</v>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%80%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>修</t>
+        </is>
+      </c>
+      <c r="B246" t="n">
+        <v>245</v>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BF%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>需</t>
+        </is>
+      </c>
+      <c r="B247" t="n">
+        <v>246</v>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%9C%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>续</t>
+        </is>
+      </c>
+      <c r="B248" t="n">
+        <v>247</v>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>宣</t>
+        </is>
+      </c>
+      <c r="B249" t="n">
+        <v>248</v>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>训</t>
+        </is>
+      </c>
+      <c r="B250" t="n">
+        <v>249</v>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AE%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>压</t>
+        </is>
+      </c>
+      <c r="B251" t="n">
+        <v>250</v>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8E%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>烟</t>
+        </is>
+      </c>
+      <c r="B252" t="n">
+        <v>251</v>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%83%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>演</t>
+        </is>
+      </c>
+      <c r="B253" t="n">
+        <v>252</v>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%BC%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>验</t>
+        </is>
+      </c>
+      <c r="B254" t="n">
+        <v>253</v>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%AA%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>羊</t>
+        </is>
+      </c>
+      <c r="B255" t="n">
+        <v>254</v>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BE%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>义</t>
+        </is>
+      </c>
+      <c r="B256" t="n">
+        <v>255</v>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B9%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>艺</t>
+        </is>
+      </c>
+      <c r="B257" t="n">
+        <v>256</v>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%89%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>议</t>
+        </is>
+      </c>
+      <c r="B258" t="n">
+        <v>257</v>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AE%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>易</t>
+        </is>
+      </c>
+      <c r="B259" t="n">
+        <v>258</v>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%98%93</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>营</t>
+        </is>
+      </c>
+      <c r="B260" t="n">
+        <v>259</v>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%90%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>赢</t>
+        </is>
+      </c>
+      <c r="B261" t="n">
+        <v>260</v>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B5%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>泳</t>
+        </is>
+      </c>
+      <c r="B262" t="n">
+        <v>261</v>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B3%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>优</t>
+        </is>
+      </c>
+      <c r="B263" t="n">
+        <v>262</v>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BC%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>邮</t>
+        </is>
+      </c>
+      <c r="B264" t="n">
+        <v>263</v>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%82%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>预</t>
+        </is>
+      </c>
+      <c r="B265" t="n">
+        <v>264</v>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A2%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>员</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>265</v>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%91%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>约</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>266</v>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BA%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>杂</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>267</v>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9D%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>造</t>
+        </is>
+      </c>
+      <c r="B269" t="n">
+        <v>268</v>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%80%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>责</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>269</v>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B4%A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>增</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>270</v>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A2%9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>展</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>271</v>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B1%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>张</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>272</v>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BC%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>章</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>273</v>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AB%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>争</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>274</v>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>整</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>275</v>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%95%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>证</t>
+        </is>
+      </c>
+      <c r="B277" t="n">
+        <v>276</v>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AF%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>支</t>
+        </is>
+      </c>
+      <c r="B278" t="n">
+        <v>277</v>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%94%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>汁</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>278</v>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B1%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>值</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>279</v>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%80%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>职</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>280</v>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%81%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>止</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>281</v>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AD%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>指</t>
+        </is>
+      </c>
+      <c r="B283" t="n">
+        <v>282</v>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8C%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>至</t>
+        </is>
+      </c>
+      <c r="B284" t="n">
+        <v>283</v>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%87%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>志</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>284</v>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BF%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>制</t>
+        </is>
+      </c>
+      <c r="B286" t="n">
+        <v>285</v>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>终</t>
+        </is>
+      </c>
+      <c r="B287" t="n">
+        <v>286</v>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>种</t>
+        </is>
+      </c>
+      <c r="B288" t="n">
+        <v>287</v>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A7%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>众</t>
+        </is>
+      </c>
+      <c r="B289" t="n">
+        <v>288</v>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BC%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>猪</t>
+        </is>
+      </c>
+      <c r="B290" t="n">
+        <v>289</v>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8C%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>注</t>
+        </is>
+      </c>
+      <c r="B291" t="n">
+        <v>290</v>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B3%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>祝</t>
+        </is>
+      </c>
+      <c r="B292" t="n">
+        <v>291</v>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A5%9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>抓</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>292</v>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8A%93</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>专</t>
+        </is>
+      </c>
+      <c r="B294" t="n">
+        <v>293</v>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%93</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>转</t>
+        </is>
+      </c>
+      <c r="B295" t="n">
+        <v>294</v>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BD%AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>状</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>295</v>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8A%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>追</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>296</v>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BF%BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>资</t>
+        </is>
+      </c>
+      <c r="B298" t="n">
+        <v>297</v>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B5%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>总</t>
+        </is>
+      </c>
+      <c r="B299" t="n">
+        <v>298</v>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%80%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>足</t>
+        </is>
+      </c>
+      <c r="B300" t="n">
+        <v>299</v>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B6%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>族</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>300</v>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%97%8F</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add HSK4 tab to HSK_words.xlsx
</commit_message>
<xml_diff>
--- a/HSK_words.xlsx
+++ b/HSK_words.xlsx
@@ -10,6 +10,7 @@
     <sheet name="HSK1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="HSK2" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="HSK3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="HSK4" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14000,4 +14001,4535 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C301"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Chữ Trung Quốc</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>阿</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%98%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>矮</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9F%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>案</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A1%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>暗</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9A%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>巴</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B7%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>摆</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%91%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>败</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B4%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>伴</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BC%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>薄</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%96%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>宝</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>抱</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8A%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>贝</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B4%9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>倍</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%80%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>笨</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AC%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>毕</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AF%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>闭</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%97%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>避</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%81%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>编</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BC%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>辩</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BE%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>冰</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%86%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>兵</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%B5</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>擦</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%93%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>财</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B4%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>操</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%93%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>测</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B5%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>抄</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8A%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>潮</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%BD%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>彻</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BD%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>沉</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B2%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>诚</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AF%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>承</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>迟</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BF%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>尺</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B0%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>冲</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%86%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>虫</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%99%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>抽</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8A%BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>窗</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AA%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>纯</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BA%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>刺</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>粗</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%B2%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>促</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BF%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>寸</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AF%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>措</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8E%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>袋</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A2%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>戴</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%88%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>担</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8B%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>淡</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B7%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>登</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%99%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>敌</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%95%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>递</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%80%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>顶</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>51</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A1%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>斗</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>52</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%96%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>豆</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>53</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B1%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>独</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>54</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8B%AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>堵</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>55</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A0%B5</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>肚</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>56</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%82%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>锻</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>57</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%94%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>恶</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>58</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%81%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>耳</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>59</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%80%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>翻</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>60</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BF%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>肥</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>61</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%82%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>纷</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>62</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BA%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>奋</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>63</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A5%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>符</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>64</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AC%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>府</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>65</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BA%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>腐</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>66</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%85%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>妇</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>67</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A6%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>附</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>68</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%99%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>盖</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>69</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9B%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>隔</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>70</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%9A%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>供</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>71</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BE%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>构</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>72</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9E%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>购</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>73</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B4%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>骨</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>74</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%AA%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>固</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>75</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9B%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>瓜</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>76</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%93%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>官</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>77</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>逛</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>78</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%80%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>归</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>79</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BD%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>裹</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>80</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A3%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>含</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>81</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>寒</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>82</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AF%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>航</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>83</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%88%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>毫</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>84</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AF%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>厚</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>85</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8E%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>乎</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>86</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B9%8E</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>呼</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>87</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%91%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>户</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>88</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%88%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>怀</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>89</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%80%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>缓</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>90</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BC%93</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>挥</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>91</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8C%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>汇</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>92</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B1%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>伙</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>93</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BC%99</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>货</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>94</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B4%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>获</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>95</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%8E%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>圾</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>96</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9C%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>激</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>97</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%BF%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>即</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>98</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8D%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>季</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>99</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AD%A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>既</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>100</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%97%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>寄</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>101</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AF%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>减</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>102</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%87%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>渐</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>103</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B8%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>江</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>104</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B1%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>奖</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>105</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A5%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>降</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>106</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%99%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>阶</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>107</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%98%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>巾</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>108</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B7%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>劲</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>109</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8A%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>禁</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>110</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A6%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>惊</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>111</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%83%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>竟</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>112</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AB%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>镜</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>113</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%95%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>究</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>114</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A9%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>居</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>115</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B1%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>局</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>116</v>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B1%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>巨</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>117</v>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B7%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>距</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>118</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B7%9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>聚</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>119</v>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%81%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>卷</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>120</v>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8D%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>均</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>121</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9D%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>棵</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>122</v>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A3%B5</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>宽</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>123</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>矿</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>124</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9F%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>扩</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>125</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>括</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>126</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8B%AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>垃</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>127</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9E%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>辣</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>128</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BE%A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>郎</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>129</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%83%8E</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>雷</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>130</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%9B%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>泪</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>131</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B3%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>厘</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>132</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8E%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>俩</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>133</v>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BF%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>炼</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>134</v>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%82%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>良</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>135</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%89%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>粮</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>136</v>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%B2%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>疗</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>137</v>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%96%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>聊</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>138</v>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%81%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>料</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>139</v>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%96%99</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>列</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>140</v>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>林</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>141</v>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9E%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>临</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>142</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>陆</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>143</v>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%99%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>律</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>144</v>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BE%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>虑</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>145</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%99%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>率</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>146</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8E%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>轮</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>147</v>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BD%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>络</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>148</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>码</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>149</v>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A0%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>帽</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>150</v>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B8%BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>梦</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>151</v>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A2%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>秘</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>152</v>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A7%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>密</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>153</v>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AF%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>免</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>154</v>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>描</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>155</v>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8F%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>摸</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>156</v>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%91%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>模</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>157</v>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A8%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>默</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>158</v>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%BB%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>闹</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>159</v>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%97%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>宁</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>160</v>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>浓</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>161</v>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B5%93</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>盘</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>162</v>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9B%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>培</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>163</v>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9F%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>婆</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>164</v>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A9%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>迫</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>165</v>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BF%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>妻</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>166</v>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A6%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>企</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>167</v>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BC%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>浅</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>168</v>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B5%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>穷</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>169</v>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A9%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>趋</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>170</v>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B6%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>趣</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>171</v>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B6%A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>圈</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>172</v>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9C%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>权</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>173</v>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9D%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>泉</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>174</v>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B3%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>却</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>175</v>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8D%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>燃</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>176</v>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%87%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>弱</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>177</v>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BC%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>伞</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>178</v>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BC%9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>扫</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>179</v>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>森</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>180</v>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A3%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>晒</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>181</v>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%99%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>闪</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>182</v>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%97%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>赏</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>183</v>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B5%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>尚</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>184</v>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B0%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>烧</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>185</v>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%83%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>申</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>186</v>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%94%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>甚</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>187</v>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%94%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>诗</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>188</v>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AF%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>施</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>189</v>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%96%BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>湿</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>190</v>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B9%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>史</t>
+        </is>
+      </c>
+      <c r="B192" t="n">
+        <v>191</v>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>士</t>
+        </is>
+      </c>
+      <c r="B193" t="n">
+        <v>192</v>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A3%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>释</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>193</v>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%87%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>守</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>194</v>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>授</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>195</v>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8E%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>售</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>196</v>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%94%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>叔</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>197</v>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>殊</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>198</v>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AE%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>暑</t>
+        </is>
+      </c>
+      <c r="B200" t="n">
+        <v>199</v>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9A%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>述</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>200</v>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BF%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>刷</t>
+        </is>
+      </c>
+      <c r="B202" t="n">
+        <v>201</v>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>帅</t>
+        </is>
+      </c>
+      <c r="B203" t="n">
+        <v>202</v>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B8%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>松</t>
+        </is>
+      </c>
+      <c r="B204" t="n">
+        <v>203</v>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9D%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>俗</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>204</v>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BF%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>塑</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>205</v>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A1%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>酸</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>206</v>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%85%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>孙</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>207</v>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AD%99</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>缩</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>208</v>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BC%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>躺</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>209</v>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BA%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>梯</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
+        <v>210</v>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A2%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>替</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>211</v>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9B%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>填</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>212</v>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A1%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>挑</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>213</v>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8C%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>贴</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>214</v>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B4%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>童</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>215</v>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AB%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>统</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>216</v>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>投</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>217</v>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8A%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>透</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>218</v>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%80%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>途</t>
+        </is>
+      </c>
+      <c r="B220" t="n">
+        <v>219</v>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%80%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>脱</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>220</v>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%84%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>袜</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>221</v>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A2%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>弯</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>222</v>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BC%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>微</t>
+        </is>
+      </c>
+      <c r="B224" t="n">
+        <v>223</v>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BE%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>维</t>
+        </is>
+      </c>
+      <c r="B225" t="n">
+        <v>224</v>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>尾</t>
+        </is>
+      </c>
+      <c r="B226" t="n">
+        <v>225</v>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B0%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>未</t>
+        </is>
+      </c>
+      <c r="B227" t="n">
+        <v>226</v>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9C%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>谓</t>
+        </is>
+      </c>
+      <c r="B228" t="n">
+        <v>227</v>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B0%93</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>稳</t>
+        </is>
+      </c>
+      <c r="B229" t="n">
+        <v>228</v>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A8%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="B230" t="n">
+        <v>229</v>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%97%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>吸</t>
+        </is>
+      </c>
+      <c r="B231" t="n">
+        <v>230</v>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>席</t>
+        </is>
+      </c>
+      <c r="B232" t="n">
+        <v>231</v>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B8%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>细</t>
+        </is>
+      </c>
+      <c r="B233" t="n">
+        <v>232</v>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>鲜</t>
+        </is>
+      </c>
+      <c r="B234" t="n">
+        <v>233</v>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%B2%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>咸</t>
+        </is>
+      </c>
+      <c r="B235" t="n">
+        <v>234</v>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%92%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>县</t>
+        </is>
+      </c>
+      <c r="B236" t="n">
+        <v>235</v>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8E%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>限</t>
+        </is>
+      </c>
+      <c r="B237" t="n">
+        <v>236</v>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%99%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>项</t>
+        </is>
+      </c>
+      <c r="B238" t="n">
+        <v>237</v>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A1%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>销</t>
+        </is>
+      </c>
+      <c r="B239" t="n">
+        <v>238</v>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%94%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>型</t>
+        </is>
+      </c>
+      <c r="B240" t="n">
+        <v>239</v>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9E%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>醒</t>
+        </is>
+      </c>
+      <c r="B241" t="n">
+        <v>240</v>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%86%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>兄</t>
+        </is>
+      </c>
+      <c r="B242" t="n">
+        <v>241</v>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>胸</t>
+        </is>
+      </c>
+      <c r="B243" t="n">
+        <v>242</v>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%83%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>秀</t>
+        </is>
+      </c>
+      <c r="B244" t="n">
+        <v>243</v>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A7%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>序</t>
+        </is>
+      </c>
+      <c r="B245" t="n">
+        <v>244</v>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BA%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>寻</t>
+        </is>
+      </c>
+      <c r="B246" t="n">
+        <v>245</v>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AF%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>迅</t>
+        </is>
+      </c>
+      <c r="B247" t="n">
+        <v>246</v>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BF%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>牙</t>
+        </is>
+      </c>
+      <c r="B248" t="n">
+        <v>247</v>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%89%99</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>亚</t>
+        </is>
+      </c>
+      <c r="B249" t="n">
+        <v>248</v>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>呀</t>
+        </is>
+      </c>
+      <c r="B250" t="n">
+        <v>249</v>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%91%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>延</t>
+        </is>
+      </c>
+      <c r="B251" t="n">
+        <v>250</v>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BB%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>严</t>
+        </is>
+      </c>
+      <c r="B252" t="n">
+        <v>251</v>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>研</t>
+        </is>
+      </c>
+      <c r="B253" t="n">
+        <v>252</v>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A0%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>盐</t>
+        </is>
+      </c>
+      <c r="B254" t="n">
+        <v>253</v>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9B%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>扬</t>
+        </is>
+      </c>
+      <c r="B255" t="n">
+        <v>254</v>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>腰</t>
+        </is>
+      </c>
+      <c r="B256" t="n">
+        <v>255</v>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%85%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>摇</t>
+        </is>
+      </c>
+      <c r="B257" t="n">
+        <v>256</v>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%91%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>叶</t>
+        </is>
+      </c>
+      <c r="B258" t="n">
+        <v>257</v>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>依</t>
+        </is>
+      </c>
+      <c r="B259" t="n">
+        <v>258</v>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BE%9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>姨</t>
+        </is>
+      </c>
+      <c r="B260" t="n">
+        <v>259</v>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A7%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>移</t>
+        </is>
+      </c>
+      <c r="B261" t="n">
+        <v>260</v>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A7%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>遗</t>
+        </is>
+      </c>
+      <c r="B262" t="n">
+        <v>261</v>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%81%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>疑</t>
+        </is>
+      </c>
+      <c r="B263" t="n">
+        <v>262</v>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%96%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>译</t>
+        </is>
+      </c>
+      <c r="B264" t="n">
+        <v>263</v>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AF%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>益</t>
+        </is>
+      </c>
+      <c r="B265" t="n">
+        <v>264</v>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9B%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>引</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>265</v>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BC%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>映</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>266</v>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%98%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>勇</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>267</v>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8B%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>幼</t>
+        </is>
+      </c>
+      <c r="B269" t="n">
+        <v>268</v>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B9%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>余</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>269</v>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BD%99</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>与</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>270</v>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%8E</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>玉</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>271</v>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8E%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>遇</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>272</v>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%81%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>圆</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>273</v>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9C%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>源</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>274</v>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%BA%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>阅</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>275</v>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%98%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>载</t>
+        </is>
+      </c>
+      <c r="B277" t="n">
+        <v>276</v>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BD%BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>赞</t>
+        </is>
+      </c>
+      <c r="B278" t="n">
+        <v>277</v>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B5%9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>则</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>278</v>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%99</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>择</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>279</v>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8B%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>战</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>280</v>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%88%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>丈</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>281</v>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>招</t>
+        </is>
+      </c>
+      <c r="B283" t="n">
+        <v>282</v>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8B%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>召</t>
+        </is>
+      </c>
+      <c r="B284" t="n">
+        <v>283</v>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>折</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>284</v>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8A%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>针</t>
+        </is>
+      </c>
+      <c r="B286" t="n">
+        <v>285</v>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%92%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>阵</t>
+        </is>
+      </c>
+      <c r="B287" t="n">
+        <v>286</v>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%98%B5</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>征</t>
+        </is>
+      </c>
+      <c r="B288" t="n">
+        <v>287</v>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BE%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>政</t>
+        </is>
+      </c>
+      <c r="B289" t="n">
+        <v>288</v>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%94%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>之</t>
+        </is>
+      </c>
+      <c r="B290" t="n">
+        <v>289</v>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B9%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>植</t>
+        </is>
+      </c>
+      <c r="B291" t="n">
+        <v>290</v>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A4%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>址</t>
+        </is>
+      </c>
+      <c r="B292" t="n">
+        <v>291</v>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9D%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>质</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>292</v>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B4%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>治</t>
+        </is>
+      </c>
+      <c r="B294" t="n">
+        <v>293</v>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B2%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>致</t>
+        </is>
+      </c>
+      <c r="B295" t="n">
+        <v>294</v>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%87%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>智</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>295</v>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%99%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>置</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>296</v>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BD%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>逐</t>
+        </is>
+      </c>
+      <c r="B298" t="n">
+        <v>297</v>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%80%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>著</t>
+        </is>
+      </c>
+      <c r="B299" t="n">
+        <v>298</v>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%91%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>综</t>
+        </is>
+      </c>
+      <c r="B300" t="n">
+        <v>299</v>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>阻</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>300</v>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%98%BB</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add HSK5 tab to HSK_words.xlsx
</commit_message>
<xml_diff>
--- a/HSK_words.xlsx
+++ b/HSK_words.xlsx
@@ -11,6 +11,7 @@
     <sheet name="HSK2" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="HSK3" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="HSK4" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="HSK5" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18532,4 +18533,4535 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C301"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Chữ Trung Quốc</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>碍</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A2%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>岸</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B2%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>拔</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8B%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>拜</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8B%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>版</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%89%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>扮</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>棒</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A3%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>悲</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%82%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>辈</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BE%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>鼻</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%BC%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>彼</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BD%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>壁</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A3%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>宾</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>饼</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A5%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>玻</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8E%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>博</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8D%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>猜</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8C%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>裁</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A3%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>册</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%86%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>叉</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>插</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8F%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>拆</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8B%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>柴</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9F%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>肠</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%82%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>尝</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B0%9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>偿</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%81%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>倡</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%80%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>乘</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B9%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>池</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B1%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>愁</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%84%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>丑</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>臭</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%87%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>厨</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8E%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>触</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A7%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>闯</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%97%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>辞</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BE%9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>聪</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%81%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>脆</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%84%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>呆</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%91%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>贷</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B4%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>胆</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%83%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>旦</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%97%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>弹</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BC%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>挡</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8C%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>德</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BE%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>丢</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>冻</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%86%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>洞</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B4%9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>毒</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AF%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>堆</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A0%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>吨</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>51</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>盾</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>52</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9B%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>朵</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>53</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9C%B5</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>躲</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>54</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BA%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>尔</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>55</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B0%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>乏</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>56</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B9%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>罚</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>57</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BD%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>繁</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>58</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%B9%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>返</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>59</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BF%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>泛</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>60</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B3%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>仿</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>61</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>疯</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>62</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%96%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>肤</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>63</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%82%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>扶</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>64</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>幅</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>65</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B9%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>辅</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>66</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BE%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>傅</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>67</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%82%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>纲</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>68</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BA%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>钢</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>69</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%92%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>糕</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>70</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%B3%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>搞</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>71</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%90%9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>革</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>72</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%9D%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>沟</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>73</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B2%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>估</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>74</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BC%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>鼓</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>75</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%BC%93</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>冠</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>76</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%86%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>鬼</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>77</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%AC%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>柜</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>78</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9F%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>滚</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>79</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%BB%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>锅</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>80</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%94%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>汗</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>81</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B1%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>豪</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>82</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B1%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>核</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>83</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A0%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>盒</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>84</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9B%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>贺</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>85</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B4%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>恨</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>86</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%81%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>猴</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>87</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8C%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>胡</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>88</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%83%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>糊</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>89</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%B3%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>虎</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>90</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%99%8E</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>滑</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>91</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%BB%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>慌</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>92</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%85%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>灰</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>93</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%81%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>恢</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>94</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%81%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>悔</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>95</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%82%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>惠</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>96</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%83%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>击</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>97</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%87%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>肌</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>98</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%82%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>辑</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>99</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BE%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>籍</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>100</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%B1%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>挤</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>101</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8C%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>夹</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>102</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>甲</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>103</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%94%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>驾</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>104</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A9%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>肩</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>105</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%82%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>艰</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>106</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%89%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>剪</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>107</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%89%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>键</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>108</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%94%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>郊</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>109</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%83%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>胶</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>110</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%83%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>戒</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>111</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%88%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>届</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>112</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B1%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>竞</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>113</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AB%9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>敬</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>114</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%95%AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>拒</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>115</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8B%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>俱</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>116</v>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BF%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>军</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>117</v>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%86%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>烤</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>118</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%83%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>颗</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>119</v>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A2%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>咳</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>120</v>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%92%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>肯</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>121</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%82%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>控</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>122</v>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8E%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>库</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>123</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BA%93</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>款</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>124</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AC%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>狂</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>125</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8B%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>亏</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>126</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>览</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>127</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A7%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>烂</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>128</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%83%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>朗</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>129</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9C%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>劳</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>130</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8A%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>梨</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>131</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A2%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>璃</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>132</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%92%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>厉</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>133</v>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8E%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>励</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>134</v>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8A%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>怜</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>135</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%80%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>帘</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>136</v>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B8%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>恋</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>137</v>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%81%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>邻</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>138</v>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%82%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>铃</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>139</v>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%93%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>龄</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>140</v>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%BE%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>令</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>141</v>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>漏</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>142</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%BC%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>逻</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>143</v>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%80%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>骂</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>144</v>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%AA%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>漫</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>145</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%BC%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>矛</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>146</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9F%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>贸</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>147</v>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B4%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>貌</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>148</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B2%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>煤</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>149</v>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%85%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>眠</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>150</v>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9C%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>秒</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>151</v>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A7%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>敏</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>152</v>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%95%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>摩</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>153</v>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%91%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>漠</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>154</v>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%BC%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>幕</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>155</v>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B9%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>奈</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>156</v>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A5%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>耐</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>157</v>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%80%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>偶</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>158</v>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%81%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>陪</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>159</v>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%99%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>赔</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>160</v>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B5%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>喷</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>161</v>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%96%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>盆</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>162</v>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9B%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>披</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>163</v>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8A%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>脾</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>164</v>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%84%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>匹</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>165</v>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8C%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>骗</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>166</v>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%AA%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>拼</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>167</v>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8B%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>频</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>168</v>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A2%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>凭</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>169</v>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%87%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>泼</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>170</v>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B3%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>葡</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>171</v>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%91%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>启</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>172</v>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>弃</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>173</v>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BC%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>签</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>174</v>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AD%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>欠</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>175</v>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AC%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>枪</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>176</v>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9E%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>抢</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>177</v>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8A%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>悄</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>178</v>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%82%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>敲</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>179</v>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%95%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>瞧</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>180</v>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9E%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>琴</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>181</v>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%90%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>勤</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>182</v>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8B%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>曲</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>183</v>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9B%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>劝</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>184</v>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8A%9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>染</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>185</v>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9F%93</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>扰</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>186</v>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>绕</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>187</v>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>忍</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>188</v>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BF%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>扔</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>189</v>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>荣</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>190</v>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%8D%A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>绒</t>
+        </is>
+      </c>
+      <c r="B192" t="n">
+        <v>191</v>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>软</t>
+        </is>
+      </c>
+      <c r="B193" t="n">
+        <v>192</v>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BD%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>润</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>193</v>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B6%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>洒</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>194</v>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B4%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>杀</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>195</v>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9D%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>傻</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>196</v>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%82%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>扇</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>197</v>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>稍</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>198</v>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A8%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>蛇</t>
+        </is>
+      </c>
+      <c r="B200" t="n">
+        <v>199</v>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%9B%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>舍</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>200</v>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%88%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>射</t>
+        </is>
+      </c>
+      <c r="B202" t="n">
+        <v>201</v>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B0%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>摄</t>
+        </is>
+      </c>
+      <c r="B203" t="n">
+        <v>202</v>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%91%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>伸</t>
+        </is>
+      </c>
+      <c r="B204" t="n">
+        <v>203</v>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BC%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>剩</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>204</v>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%89%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>拾</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>205</v>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8B%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>驶</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>206</v>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A9%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>饰</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>207</v>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A5%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>柿</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>208</v>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9F%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>寿</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>209</v>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AF%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>瘦</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
+        <v>210</v>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%98%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>蔬</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>211</v>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%94%AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>鼠</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>212</v>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%BC%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>摔</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>213</v>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%91%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>硕</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>214</v>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A1%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>私</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>215</v>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A7%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>搜</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>216</v>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%90%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>肃</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>217</v>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%82%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>宿</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>218</v>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>碎</t>
+        </is>
+      </c>
+      <c r="B220" t="n">
+        <v>219</v>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A2%8E</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>损</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>220</v>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8D%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>索</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>221</v>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%B4%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>锁</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>222</v>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%94%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>抬</t>
+        </is>
+      </c>
+      <c r="B224" t="n">
+        <v>223</v>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8A%AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>坦</t>
+        </is>
+      </c>
+      <c r="B225" t="n">
+        <v>224</v>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9D%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>逃</t>
+        </is>
+      </c>
+      <c r="B226" t="n">
+        <v>225</v>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%80%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>桃</t>
+        </is>
+      </c>
+      <c r="B227" t="n">
+        <v>226</v>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A1%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>萄</t>
+        </is>
+      </c>
+      <c r="B228" t="n">
+        <v>227</v>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%90%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>厅</t>
+        </is>
+      </c>
+      <c r="B229" t="n">
+        <v>228</v>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8E%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>偷</t>
+        </is>
+      </c>
+      <c r="B230" t="n">
+        <v>229</v>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%81%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>吐</t>
+        </is>
+      </c>
+      <c r="B231" t="n">
+        <v>230</v>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>兔</t>
+        </is>
+      </c>
+      <c r="B232" t="n">
+        <v>231</v>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>托</t>
+        </is>
+      </c>
+      <c r="B233" t="n">
+        <v>232</v>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>违</t>
+        </is>
+      </c>
+      <c r="B234" t="n">
+        <v>233</v>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BF%9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>唯</t>
+        </is>
+      </c>
+      <c r="B235" t="n">
+        <v>234</v>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%94%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>委</t>
+        </is>
+      </c>
+      <c r="B236" t="n">
+        <v>235</v>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A7%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>胃</t>
+        </is>
+      </c>
+      <c r="B237" t="n">
+        <v>236</v>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%83%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>慰</t>
+        </is>
+      </c>
+      <c r="B238" t="n">
+        <v>237</v>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%85%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>卧</t>
+        </is>
+      </c>
+      <c r="B239" t="n">
+        <v>238</v>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8D%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>污</t>
+        </is>
+      </c>
+      <c r="B240" t="n">
+        <v>239</v>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B1%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>夕</t>
+        </is>
+      </c>
+      <c r="B241" t="n">
+        <v>240</v>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>析</t>
+        </is>
+      </c>
+      <c r="B242" t="n">
+        <v>241</v>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9E%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>悉</t>
+        </is>
+      </c>
+      <c r="B243" t="n">
+        <v>242</v>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%82%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>惜</t>
+        </is>
+      </c>
+      <c r="B244" t="n">
+        <v>243</v>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%83%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>吓</t>
+        </is>
+      </c>
+      <c r="B245" t="n">
+        <v>244</v>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%93</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>闲</t>
+        </is>
+      </c>
+      <c r="B246" t="n">
+        <v>245</v>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%97%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>献</t>
+        </is>
+      </c>
+      <c r="B247" t="n">
+        <v>246</v>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8C%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>详</t>
+        </is>
+      </c>
+      <c r="B248" t="n">
+        <v>247</v>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AF%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>享</t>
+        </is>
+      </c>
+      <c r="B249" t="n">
+        <v>248</v>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>歇</t>
+        </is>
+      </c>
+      <c r="B250" t="n">
+        <v>249</v>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AD%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>协</t>
+        </is>
+      </c>
+      <c r="B251" t="n">
+        <v>250</v>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8D%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>斜</t>
+        </is>
+      </c>
+      <c r="B252" t="n">
+        <v>251</v>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%96%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>辛</t>
+        </is>
+      </c>
+      <c r="B253" t="n">
+        <v>252</v>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BE%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>欣</t>
+        </is>
+      </c>
+      <c r="B254" t="n">
+        <v>253</v>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AC%A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>雄</t>
+        </is>
+      </c>
+      <c r="B255" t="n">
+        <v>254</v>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%9B%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>熊</t>
+        </is>
+      </c>
+      <c r="B256" t="n">
+        <v>255</v>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%86%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>虚</t>
+        </is>
+      </c>
+      <c r="B257" t="n">
+        <v>256</v>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%99%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>询</t>
+        </is>
+      </c>
+      <c r="B258" t="n">
+        <v>257</v>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AF%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>押</t>
+        </is>
+      </c>
+      <c r="B259" t="n">
+        <v>258</v>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8A%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>鸭</t>
+        </is>
+      </c>
+      <c r="B260" t="n">
+        <v>259</v>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%B8%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>厌</t>
+        </is>
+      </c>
+      <c r="B261" t="n">
+        <v>260</v>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8E%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>艳</t>
+        </is>
+      </c>
+      <c r="B262" t="n">
+        <v>261</v>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%89%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>央</t>
+        </is>
+      </c>
+      <c r="B263" t="n">
+        <v>262</v>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>邀</t>
+        </is>
+      </c>
+      <c r="B264" t="n">
+        <v>263</v>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%82%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>咬</t>
+        </is>
+      </c>
+      <c r="B265" t="n">
+        <v>264</v>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%92%AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>乙</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>265</v>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B9%99</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>忆</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>266</v>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BF%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>谊</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>267</v>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B0%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>饮</t>
+        </is>
+      </c>
+      <c r="B269" t="n">
+        <v>268</v>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A5%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>硬</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>269</v>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A1%AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>拥</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>270</v>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8B%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>幽</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>271</v>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B9%BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>尤</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>272</v>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B0%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>犹</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>273</v>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8A%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>羽</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>274</v>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BE%BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>域</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>275</v>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9F%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>豫</t>
+        </is>
+      </c>
+      <c r="B277" t="n">
+        <v>276</v>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B1%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>怨</t>
+        </is>
+      </c>
+      <c r="B278" t="n">
+        <v>277</v>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%80%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>灾</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>278</v>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%81%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>仔</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>279</v>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>暂</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>280</v>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9A%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>糟</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>281</v>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%B3%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>赠</t>
+        </is>
+      </c>
+      <c r="B283" t="n">
+        <v>282</v>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B5%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>摘</t>
+        </is>
+      </c>
+      <c r="B284" t="n">
+        <v>283</v>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%91%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>涨</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>284</v>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B6%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>掌</t>
+        </is>
+      </c>
+      <c r="B286" t="n">
+        <v>285</v>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8E%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>珍</t>
+        </is>
+      </c>
+      <c r="B287" t="n">
+        <v>286</v>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8F%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>诊</t>
+        </is>
+      </c>
+      <c r="B288" t="n">
+        <v>287</v>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AF%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>振</t>
+        </is>
+      </c>
+      <c r="B289" t="n">
+        <v>288</v>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8C%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>震</t>
+        </is>
+      </c>
+      <c r="B290" t="n">
+        <v>289</v>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%9C%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>挣</t>
+        </is>
+      </c>
+      <c r="B291" t="n">
+        <v>290</v>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8C%A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>织</t>
+        </is>
+      </c>
+      <c r="B292" t="n">
+        <v>291</v>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>执</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>292</v>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>珠</t>
+        </is>
+      </c>
+      <c r="B294" t="n">
+        <v>293</v>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8F%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>竹</t>
+        </is>
+      </c>
+      <c r="B295" t="n">
+        <v>294</v>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AB%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>筑</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>295</v>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AD%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>撞</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>296</v>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%92%9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>紫</t>
+        </is>
+      </c>
+      <c r="B298" t="n">
+        <v>297</v>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%B4%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>醉</t>
+        </is>
+      </c>
+      <c r="B299" t="n">
+        <v>298</v>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%86%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>尊</t>
+        </is>
+      </c>
+      <c r="B300" t="n">
+        <v>299</v>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B0%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>遵</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>300</v>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%81%B5</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add HSK6 tab to HSK_words.xlsx
</commit_message>
<xml_diff>
--- a/HSK_words.xlsx
+++ b/HSK_words.xlsx
@@ -12,6 +12,7 @@
     <sheet name="HSK3" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="HSK4" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="HSK5" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="HSK6" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23064,4 +23065,4535 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C301"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Chữ Trung Quốc</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>挨</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8C%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>傲</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%82%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>罢</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BD%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>榜</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A6%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>傍</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%82%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>胞</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%83%9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>暴</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9A%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>爆</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%88%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>奔</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A5%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>逼</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%80%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>扁</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>拨</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8B%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>波</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B3%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>捕</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8D%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>踩</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B8%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>残</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AE%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>惨</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%83%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>仓</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%93</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>藏</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%97%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>厕</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8E%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>侧</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BE%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>策</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AD%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>昌</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%98%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>畅</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%95%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>炒</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>25</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%82%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>撤</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>26</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%92%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>撑</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>27</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%92%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>崇</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>28</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B4%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>宠</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>29</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>储</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>30</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%82%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>串</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>31</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>醋</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>32</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%86%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>搭</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%90%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>诞</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AF%9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>党</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>档</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A1%A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>岛</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B2%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>蹈</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>38</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B9%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>盗</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>39</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9B%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>滴</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>40</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%BB%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>抵</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>41</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8A%B5</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>帝</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>42</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B8%9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>吊</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>43</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>跌</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>44</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B7%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>督</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9D%A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>赌</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B5%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>渡</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>47</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B8%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>端</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>48</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AB%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>蹲</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>49</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B9%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>夺</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>50</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>额</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>51</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A2%9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>恩</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>52</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%81%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>番</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>53</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%95%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>凡</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>54</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%87%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>犯</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>55</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8A%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>肺</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>56</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%82%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>废</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>57</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BA%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>氛</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>58</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B0%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>粉</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>59</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%B2%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>愤</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>60</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%84%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>峰</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>61</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B3%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>锋</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>62</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%94%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>奉</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>63</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A5%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>佛</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>64</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BD%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>浮</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>65</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B5%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>副</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>66</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%89%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>肝</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>67</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%82%9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>杆</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>68</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9D%86</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>岗</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>69</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B2%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>港</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>70</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B8%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>稿</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>71</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A8%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>攻</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>72</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%94%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>宫</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>73</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>巩</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>74</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B7%A9</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>贡</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>75</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B4%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>孤</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>76</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AD%A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>谷</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>77</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B0%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>股</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>78</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%82%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>刮</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>79</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>拐</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>80</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8B%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>贯</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>81</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B4%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>轨</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>82</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BD%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>跪</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>83</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B7%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>憾</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>84</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%86%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>耗</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>85</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%80%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>狠</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>86</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8B%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>横</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>87</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A8%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>衡</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>88</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A1%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>宏</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>89</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>洪</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>90</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B4%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>壶</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>91</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A3%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>幻</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>92</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B9%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>患</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>93</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%82%A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>皇</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>94</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9A%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>辉</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>95</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BE%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>毁</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>96</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AF%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>绘</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>97</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>慧</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>98</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%85%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>昏</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>99</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%98%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>混</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>100</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B7%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>吉</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>101</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>疾</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>102</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%96%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>佳</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>103</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BD%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>嘉</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>104</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%98%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>尖</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>105</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B0%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>监</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>106</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9B%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>捡</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>107</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8D%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>剑</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>108</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%89%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>舰</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>109</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%88%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>践</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>110</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B7%B5</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>鉴</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>111</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%89%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>箭</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>112</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AE%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>酱</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>113</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%85%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>骄</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>114</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%AA%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>焦</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>115</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%84%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>揭</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>116</v>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8F%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>杰</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>117</v>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9D%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>洁</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>118</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B4%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>截</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>119</v>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%88%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>井</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>120</v>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>径</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>121</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BE%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>纠</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>122</v>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BA%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>捐</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>123</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8D%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>菌</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>124</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%8F%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>刊</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>125</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>抗</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>126</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8A%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>扣</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>127</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>酷</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>128</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%85%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>跨</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>129</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B7%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>阔</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>130</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%98%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>啦</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>131</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%95%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>赖</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>132</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B5%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>栏</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>133</v>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A0%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>懒</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>134</v>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%87%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>牢</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>135</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%89%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>梁</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>136</v>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A2%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>谅</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>137</v>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B0%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>裂</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>138</v>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A3%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>灵</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>139</v>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%81%B5</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>炉</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>140</v>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%82%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>露</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>141</v>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%9C%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>略</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>142</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%95%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>嘛</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>143</v>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%98%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>埋</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>144</v>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9F%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>麦</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>145</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%BA%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>馒</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>146</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A6%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>盲</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>147</v>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9B%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>梅</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>148</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A2%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>蒙</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>149</v>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%92%99</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>盟</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>150</v>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9B%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>猛</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>151</v>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8C%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>棉</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>152</v>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A3%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>妙</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>153</v>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A6%99</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>灭</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>154</v>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%81%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>膜</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>155</v>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%86%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>磨</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>156</v>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A3%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>墨</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>157</v>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A2%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>谋</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>158</v>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B0%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>墓</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>159</v>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A2%93</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>纳</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>160</v>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BA%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>泥</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>161</v>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B3%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>扭</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>162</v>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>怒</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>163</v>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%80%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>诺</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>164</v>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AF%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>盼</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>165</v>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9B%BC</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>泡</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>166</v>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B3%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>炮</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>167</v>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%82%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>偏</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>168</v>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%81%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>贫</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>169</v>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B4%AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>聘</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>170</v>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%81%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>屏</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>171</v>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B1%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>坡</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>172</v>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9D%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>扑</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>173</v>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%91</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>铺</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>174</v>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%93%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>欺</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>175</v>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AC%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>旗</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>176</v>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%97%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>恰</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>177</v>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%81%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>迁</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>178</v>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BF%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>牵</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>179</v>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%89%B5</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>铅</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>180</v>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%93%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>谦</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>181</v>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B0%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>潜</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>182</v>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%BD%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>歉</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>183</v>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AD%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>茄</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>184</v>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%8C%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>侵</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>185</v>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BE%B5</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>倾</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>186</v>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%80%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>渠</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>187</v>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B8%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>券</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>188</v>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>融</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>189</v>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%9E%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>乳</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>190</v>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B9%B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>若</t>
+        </is>
+      </c>
+      <c r="B192" t="n">
+        <v>191</v>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%8B%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>塞</t>
+        </is>
+      </c>
+      <c r="B193" t="n">
+        <v>192</v>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A1%9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>丧</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>193</v>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>勺</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>194</v>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8B%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>舌</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>195</v>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%88%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>涉</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>196</v>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B6%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>审</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>197</v>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>牲</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>198</v>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%89%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>圣</t>
+        </is>
+      </c>
+      <c r="B200" t="n">
+        <v>199</v>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9C%A3</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>盛</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>200</v>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9B%9B</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>薯</t>
+        </is>
+      </c>
+      <c r="B202" t="n">
+        <v>201</v>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%96%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>爽</t>
+        </is>
+      </c>
+      <c r="B203" t="n">
+        <v>202</v>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%88%BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>税</t>
+        </is>
+      </c>
+      <c r="B204" t="n">
+        <v>203</v>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A8%8E</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>寺</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>204</v>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AF%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>苏</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>205</v>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%8B%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>素</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>206</v>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%B4%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>塔</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>207</v>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A1%94</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>踏</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>208</v>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B8%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>叹</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>209</v>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%B9</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>探</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
+        <v>210</v>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8E%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>趟</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>211</v>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B6%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>掏</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>212</v>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8E%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>踢</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>213</v>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B8%A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>添</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>214</v>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B7%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>田</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>215</v>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%94%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>铜</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>216</v>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%93%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>徒</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>217</v>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BE%92</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>吞</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>218</v>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%9E</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>拖</t>
+        </is>
+      </c>
+      <c r="B220" t="n">
+        <v>219</v>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8B%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>挖</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>220</v>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8C%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>娃</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>221</v>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A8%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>哇</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>222</v>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%93%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>湾</t>
+        </is>
+      </c>
+      <c r="B224" t="n">
+        <v>223</v>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B9%BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>顽</t>
+        </is>
+      </c>
+      <c r="B225" t="n">
+        <v>224</v>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A1%BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>亡</t>
+        </is>
+      </c>
+      <c r="B226" t="n">
+        <v>225</v>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%A1</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>旺</t>
+        </is>
+      </c>
+      <c r="B227" t="n">
+        <v>226</v>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%97%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>威</t>
+        </is>
+      </c>
+      <c r="B228" t="n">
+        <v>227</v>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A8%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>乌</t>
+        </is>
+      </c>
+      <c r="B229" t="n">
+        <v>228</v>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B9%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>伍</t>
+        </is>
+      </c>
+      <c r="B230" t="n">
+        <v>229</v>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BC%8D</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>悟</t>
+        </is>
+      </c>
+      <c r="B231" t="n">
+        <v>230</v>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%82%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>牺</t>
+        </is>
+      </c>
+      <c r="B232" t="n">
+        <v>231</v>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%89%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>嫌</t>
+        </is>
+      </c>
+      <c r="B233" t="n">
+        <v>232</v>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AB%8C</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>陷</t>
+        </is>
+      </c>
+      <c r="B234" t="n">
+        <v>233</v>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%99%B7</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>祥</t>
+        </is>
+      </c>
+      <c r="B235" t="n">
+        <v>234</v>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A5%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>晓</t>
+        </is>
+      </c>
+      <c r="B236" t="n">
+        <v>235</v>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%99%93</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>胁</t>
+        </is>
+      </c>
+      <c r="B237" t="n">
+        <v>236</v>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%83%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>谐</t>
+        </is>
+      </c>
+      <c r="B238" t="n">
+        <v>237</v>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B0%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>械</t>
+        </is>
+      </c>
+      <c r="B239" t="n">
+        <v>238</v>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A2%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>薪</t>
+        </is>
+      </c>
+      <c r="B240" t="n">
+        <v>239</v>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%96%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>凶</t>
+        </is>
+      </c>
+      <c r="B241" t="n">
+        <v>240</v>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%87%B6</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>袖</t>
+        </is>
+      </c>
+      <c r="B242" t="n">
+        <v>241</v>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A2%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>绪</t>
+        </is>
+      </c>
+      <c r="B243" t="n">
+        <v>242</v>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>悬</t>
+        </is>
+      </c>
+      <c r="B244" t="n">
+        <v>243</v>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%82%AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>旋</t>
+        </is>
+      </c>
+      <c r="B245" t="n">
+        <v>244</v>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%97%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>循</t>
+        </is>
+      </c>
+      <c r="B246" t="n">
+        <v>245</v>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BE%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>讯</t>
+        </is>
+      </c>
+      <c r="B247" t="n">
+        <v>246</v>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AE%AF</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>炎</t>
+        </is>
+      </c>
+      <c r="B248" t="n">
+        <v>247</v>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%82%8E</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>沿</t>
+        </is>
+      </c>
+      <c r="B249" t="n">
+        <v>248</v>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B2%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>宴</t>
+        </is>
+      </c>
+      <c r="B250" t="n">
+        <v>249</v>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>洋</t>
+        </is>
+      </c>
+      <c r="B251" t="n">
+        <v>250</v>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B4%8B</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>仰</t>
+        </is>
+      </c>
+      <c r="B252" t="n">
+        <v>251</v>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%B0</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>氧</t>
+        </is>
+      </c>
+      <c r="B253" t="n">
+        <v>252</v>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B0%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>耀</t>
+        </is>
+      </c>
+      <c r="B254" t="n">
+        <v>253</v>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%80%80</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>野</t>
+        </is>
+      </c>
+      <c r="B255" t="n">
+        <v>254</v>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%87%8E</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>液</t>
+        </is>
+      </c>
+      <c r="B256" t="n">
+        <v>255</v>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B6%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>仪</t>
+        </is>
+      </c>
+      <c r="B257" t="n">
+        <v>256</v>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>异</t>
+        </is>
+      </c>
+      <c r="B258" t="n">
+        <v>257</v>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BC%82</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>隐</t>
+        </is>
+      </c>
+      <c r="B259" t="n">
+        <v>258</v>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%9A%90</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>忧</t>
+        </is>
+      </c>
+      <c r="B260" t="n">
+        <v>259</v>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BF%A7</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>娱</t>
+        </is>
+      </c>
+      <c r="B261" t="n">
+        <v>260</v>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A8%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>愉</t>
+        </is>
+      </c>
+      <c r="B262" t="n">
+        <v>261</v>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%84%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>予</t>
+        </is>
+      </c>
+      <c r="B263" t="n">
+        <v>262</v>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%88</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>宇</t>
+        </is>
+      </c>
+      <c r="B264" t="n">
+        <v>263</v>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>欲</t>
+        </is>
+      </c>
+      <c r="B265" t="n">
+        <v>264</v>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AC%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>誉</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>265</v>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AA%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>援</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>266</v>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8F%B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>缘</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>267</v>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BC%98</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>跃</t>
+        </is>
+      </c>
+      <c r="B269" t="n">
+        <v>268</v>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B7%83</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>晕</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>269</v>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%99%95</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>允</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>270</v>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%81</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>遭</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>271</v>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%81%AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>扎</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>272</v>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%8E</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>炸</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>273</v>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%82%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>宅</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>274</v>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%85</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>债</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>275</v>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%80%BA</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>账</t>
+        </is>
+      </c>
+      <c r="B277" t="n">
+        <v>276</v>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B4%A6</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>障</t>
+        </is>
+      </c>
+      <c r="B278" t="n">
+        <v>277</v>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%9A%9C</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>哲</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>278</v>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%93%B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>镇</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>279</v>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%95%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>症</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>280</v>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%97%87</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>枝</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>281</v>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9E%9D</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>殖</t>
+        </is>
+      </c>
+      <c r="B283" t="n">
+        <v>282</v>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AE%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>忠</t>
+        </is>
+      </c>
+      <c r="B284" t="n">
+        <v>283</v>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BF%A0</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>肿</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>284</v>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%82%BF</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>粥</t>
+        </is>
+      </c>
+      <c r="B286" t="n">
+        <v>285</v>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%B2%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>诸</t>
+        </is>
+      </c>
+      <c r="B287" t="n">
+        <v>286</v>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AF%B8</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>煮</t>
+        </is>
+      </c>
+      <c r="B288" t="n">
+        <v>287</v>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%85%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>驻</t>
+        </is>
+      </c>
+      <c r="B289" t="n">
+        <v>288</v>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A9%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>柱</t>
+        </is>
+      </c>
+      <c r="B290" t="n">
+        <v>289</v>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9F%B1</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>赚</t>
+        </is>
+      </c>
+      <c r="B291" t="n">
+        <v>290</v>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B5%9A</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>庄</t>
+        </is>
+      </c>
+      <c r="B292" t="n">
+        <v>291</v>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BA%84</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>壮</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>292</v>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A3%AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>捉</t>
+        </is>
+      </c>
+      <c r="B294" t="n">
+        <v>293</v>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8D%89</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>咨</t>
+        </is>
+      </c>
+      <c r="B295" t="n">
+        <v>294</v>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%92%A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>宗</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>295</v>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%97</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>纵</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>296</v>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BA%B5</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>奏</t>
+        </is>
+      </c>
+      <c r="B298" t="n">
+        <v>297</v>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A5%8F</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>祖</t>
+        </is>
+      </c>
+      <c r="B299" t="n">
+        <v>298</v>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A5%96</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>钻</t>
+        </is>
+      </c>
+      <c r="B300" t="n">
+        <v>299</v>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%92%BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>罪</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>300</v>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BD%AA</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>